<commit_message>
Snapshot of the finished demo run (Oct 12, 2026)
</commit_message>
<xml_diff>
--- a/data/download/model_forecast.xlsx
+++ b/data/download/model_forecast.xlsx
@@ -838,10 +838,10 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>0.37</v>
+        <v>0.353</v>
       </c>
       <c r="C11" s="9" t="n">
-        <v>0.38</v>
+        <v>0.373</v>
       </c>
       <c r="D11" s="9" t="n">
         <v>0.39</v>
@@ -893,7 +893,7 @@
         <v>0.025</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>0.027</v>
+        <v>0.0275</v>
       </c>
       <c r="D13" s="9" t="n">
         <v>0.03</v>
@@ -916,10 +916,10 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.46</v>
+        <v>0.4485</v>
       </c>
       <c r="C14" s="9" t="n">
-        <v>0.45</v>
+        <v>0.4455</v>
       </c>
       <c r="D14" s="9" t="n">
         <v>0.445</v>
@@ -1501,7 +1501,7 @@
         <v>89.023</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F7" s="10">
         <f>IF(COUNT(B7:E7)&lt;4,"",(B12-SUM(B9:E9))/F8)</f>
@@ -1582,7 +1582,7 @@
       </c>
       <c r="E10" s="12" t="inlineStr">
         <is>
-          <t>nvda-2026-08-26-release</t>
+          <t>channel-q4-slip</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16">
@@ -1690,11 +1690,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>372</v>
+        <v>376</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>street-oct2026</t>
+          <t>broker-oct2026</t>
         </is>
       </c>
     </row>
@@ -1709,7 +1709,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>street-oct2026</t>
+          <t>broker-oct2026</t>
         </is>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2320,6 +2320,197 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Inputs!C11</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.373</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Dated synthetic calendar-Q4-to-Q1 deferral allegations change timing odds despite unverified respondent independence and customer IDs. System value $12-15bn x reported 70% NVIDIA is $8.4-10.5bn branded rack value, not NVIDIA revenue. Size direct total-NVIDIA base haircut at about $3.15bn: $13.5bn midpoint x70% x assumed 2/3 supplier content x50% net confidence/recognition-shift weight; bear about $7.56bn uses 80% content and full realization. These conversion/weights are judgment, not disclosed BOM or probabilities. Base mix 38%-&gt;37.3% and NVDA Big4 concentration 45%-&gt;44.55% jointly calibrate ~$3.19bn direct global hit while keeping non-Big4 NVDA dollars approximately unchanged; do not gross a customer-specific loss up by 1/concentration. Bear mix 37%-&gt;35.3%, concentration46%-&gt;44.85% give ~$7.55bn hit. Base AMD split2.7%-&gt;2.75% recalibrates unchanged ~$14bn GPU anchor after shared-mix change; no claim of competitive share gain. Hold all company capex estimates pending IDs/measure reconciliation; lower realized accelerator mix is a provisional timing proxy assuming other infrastructure/prepaid/offset deliveries can fill current budgets, not a measured cash-capex cut. If named cash cuts are confirmed replace/reconcile the proxy to avoid double counting. Hold NVIDIA competitive split and bull. Separate quarterly tool revises Q3DC103-&gt;102 and own Q4DC128-&gt;127: roughly even original Oct-Dec and new Jan-Mar placement makes expected ~$1.05bn net hit to each fiscal quarter; January remains FYQ4.</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>channel-q4-slip, channel-oct2026, web-b93e425ae9, web-81e32d74b6, web-454ed8f95a, meta-2026-07-29-release, nvda-2026-08-26-release, amd-2026-08-04-release</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Inputs!C14</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0.4455</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Dated synthetic calendar-Q4-to-Q1 deferral allegations change timing odds despite unverified respondent independence and customer IDs. System value $12-15bn x reported 70% NVIDIA is $8.4-10.5bn branded rack value, not NVIDIA revenue. Size direct total-NVIDIA base haircut at about $3.15bn: $13.5bn midpoint x70% x assumed 2/3 supplier content x50% net confidence/recognition-shift weight; bear about $7.56bn uses 80% content and full realization. These conversion/weights are judgment, not disclosed BOM or probabilities. Base mix 38%-&gt;37.3% and NVDA Big4 concentration 45%-&gt;44.55% jointly calibrate ~$3.19bn direct global hit while keeping non-Big4 NVDA dollars approximately unchanged; do not gross a customer-specific loss up by 1/concentration. Bear mix 37%-&gt;35.3%, concentration46%-&gt;44.85% give ~$7.55bn hit. Base AMD split2.7%-&gt;2.75% recalibrates unchanged ~$14bn GPU anchor after shared-mix change; no claim of competitive share gain. Hold all company capex estimates pending IDs/measure reconciliation; lower realized accelerator mix is a provisional timing proxy assuming other infrastructure/prepaid/offset deliveries can fill current budgets, not a measured cash-capex cut. If named cash cuts are confirmed replace/reconcile the proxy to avoid double counting. Hold NVIDIA competitive split and bull. Separate quarterly tool revises Q3DC103-&gt;102 and own Q4DC128-&gt;127: roughly even original Oct-Dec and new Jan-Mar placement makes expected ~$1.05bn net hit to each fiscal quarter; January remains FYQ4.</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>channel-q4-slip, channel-oct2026, web-b93e425ae9, web-81e32d74b6, web-454ed8f95a, meta-2026-07-29-release, nvda-2026-08-26-release, amd-2026-08-04-release</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Inputs!C13</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.0275</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Dated synthetic calendar-Q4-to-Q1 deferral allegations change timing odds despite unverified respondent independence and customer IDs. System value $12-15bn x reported 70% NVIDIA is $8.4-10.5bn branded rack value, not NVIDIA revenue. Size direct total-NVIDIA base haircut at about $3.15bn: $13.5bn midpoint x70% x assumed 2/3 supplier content x50% net confidence/recognition-shift weight; bear about $7.56bn uses 80% content and full realization. These conversion/weights are judgment, not disclosed BOM or probabilities. Base mix 38%-&gt;37.3% and NVDA Big4 concentration 45%-&gt;44.55% jointly calibrate ~$3.19bn direct global hit while keeping non-Big4 NVDA dollars approximately unchanged; do not gross a customer-specific loss up by 1/concentration. Bear mix 37%-&gt;35.3%, concentration46%-&gt;44.85% give ~$7.55bn hit. Base AMD split2.7%-&gt;2.75% recalibrates unchanged ~$14bn GPU anchor after shared-mix change; no claim of competitive share gain. Hold all company capex estimates pending IDs/measure reconciliation; lower realized accelerator mix is a provisional timing proxy assuming other infrastructure/prepaid/offset deliveries can fill current budgets, not a measured cash-capex cut. If named cash cuts are confirmed replace/reconcile the proxy to avoid double counting. Hold NVIDIA competitive split and bull. Separate quarterly tool revises Q3DC103-&gt;102 and own Q4DC128-&gt;127: roughly even original Oct-Dec and new Jan-Mar placement makes expected ~$1.05bn net hit to each fiscal quarter; January remains FYQ4.</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>channel-q4-slip, channel-oct2026, web-b93e425ae9, web-81e32d74b6, web-454ed8f95a, meta-2026-07-29-release, nvda-2026-08-26-release, amd-2026-08-04-release</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Inputs!B11</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.353</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Dated synthetic calendar-Q4-to-Q1 deferral allegations change timing odds despite unverified respondent independence and customer IDs. System value $12-15bn x reported 70% NVIDIA is $8.4-10.5bn branded rack value, not NVIDIA revenue. Size direct total-NVIDIA base haircut at about $3.15bn: $13.5bn midpoint x70% x assumed 2/3 supplier content x50% net confidence/recognition-shift weight; bear about $7.56bn uses 80% content and full realization. These conversion/weights are judgment, not disclosed BOM or probabilities. Base mix 38%-&gt;37.3% and NVDA Big4 concentration 45%-&gt;44.55% jointly calibrate ~$3.19bn direct global hit while keeping non-Big4 NVDA dollars approximately unchanged; do not gross a customer-specific loss up by 1/concentration. Bear mix 37%-&gt;35.3%, concentration46%-&gt;44.85% give ~$7.55bn hit. Base AMD split2.7%-&gt;2.75% recalibrates unchanged ~$14bn GPU anchor after shared-mix change; no claim of competitive share gain. Hold all company capex estimates pending IDs/measure reconciliation; lower realized accelerator mix is a provisional timing proxy assuming other infrastructure/prepaid/offset deliveries can fill current budgets, not a measured cash-capex cut. If named cash cuts are confirmed replace/reconcile the proxy to avoid double counting. Hold NVIDIA competitive split and bull. Separate quarterly tool revises Q3DC103-&gt;102 and own Q4DC128-&gt;127: roughly even original Oct-Dec and new Jan-Mar placement makes expected ~$1.05bn net hit to each fiscal quarter; January remains FYQ4.</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>channel-q4-slip, channel-oct2026, web-b93e425ae9, web-81e32d74b6, web-454ed8f95a, meta-2026-07-29-release, nvda-2026-08-26-release, amd-2026-08-04-release</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Inputs!B14</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.4485</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Dated synthetic calendar-Q4-to-Q1 deferral allegations change timing odds despite unverified respondent independence and customer IDs. System value $12-15bn x reported 70% NVIDIA is $8.4-10.5bn branded rack value, not NVIDIA revenue. Size direct total-NVIDIA base haircut at about $3.15bn: $13.5bn midpoint x70% x assumed 2/3 supplier content x50% net confidence/recognition-shift weight; bear about $7.56bn uses 80% content and full realization. These conversion/weights are judgment, not disclosed BOM or probabilities. Base mix 38%-&gt;37.3% and NVDA Big4 concentration 45%-&gt;44.55% jointly calibrate ~$3.19bn direct global hit while keeping non-Big4 NVDA dollars approximately unchanged; do not gross a customer-specific loss up by 1/concentration. Bear mix 37%-&gt;35.3%, concentration46%-&gt;44.85% give ~$7.55bn hit. Base AMD split2.7%-&gt;2.75% recalibrates unchanged ~$14bn GPU anchor after shared-mix change; no claim of competitive share gain. Hold all company capex estimates pending IDs/measure reconciliation; lower realized accelerator mix is a provisional timing proxy assuming other infrastructure/prepaid/offset deliveries can fill current budgets, not a measured cash-capex cut. If named cash cuts are confirmed replace/reconcile the proxy to avoid double counting. Hold NVIDIA competitive split and bull. Separate quarterly tool revises Q3DC103-&gt;102 and own Q4DC128-&gt;127: roughly even original Oct-Dec and new Jan-Mar placement makes expected ~$1.05bn net hit to each fiscal quarter; January remains FYQ4.</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>channel-q4-slip, channel-oct2026, web-b93e425ae9, web-81e32d74b6, web-454ed8f95a, meta-2026-07-29-release, nvda-2026-08-26-release, amd-2026-08-04-release</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Quarters!E7</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>103</v>
+      </c>
+      <c r="D26" t="n">
+        <v>102</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Revise unreported Q3 FY27 Data Center 103-&gt;102 and own Q4 FY27 128-&gt;127 on dated Q4 CY2026 rack deferrals. Direct expected calendar revenue shift ~$3.15bn is judgment from branded-value/content/net-realization assumptions. Assume original shifted supplier revenue roughly evenly in Oct/Nov/Dec and receipts Jan/Feb/Mar: Q3 loses October ~$1.05bn; FYQ4 loses Nov/Dec ~$2.10bn but gains January ~$1.05bn, net loss ~$1.05bn, rounded to $1bn each. These month allocations are estimates, not vendor detail. New Q3 total109.5 less Edge7.5 is a1.4% beat vs108 guide. Expected Nov18 report remains unconfirmed. Filing-exact reported quarters unchanged. New top-down annual371.4301 implies FYQ4 126.5847 at revised Q3 102; own127 yields monthly bridge371.707. Fixed monthly weights cannot fully measure January redistribution; saved formulas/application recalculation, not pre-decision snapshot diagnostics, govern.</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>channel-q4-slip</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-12</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Quarters!B15</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>128</v>
+      </c>
+      <c r="D27" t="n">
+        <v>127</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Revise unreported Q3 FY27 Data Center 103-&gt;102 and own Q4 FY27 128-&gt;127 on dated Q4 CY2026 rack deferrals. Direct expected calendar revenue shift ~$3.15bn is judgment from branded-value/content/net-realization assumptions. Assume original shifted supplier revenue roughly evenly in Oct/Nov/Dec and receipts Jan/Feb/Mar: Q3 loses October ~$1.05bn; FYQ4 loses Nov/Dec ~$2.10bn but gains January ~$1.05bn, net loss ~$1.05bn, rounded to $1bn each. These month allocations are estimates, not vendor detail. New Q3 total109.5 less Edge7.5 is a1.4% beat vs108 guide. Expected Nov18 report remains unconfirmed. Filing-exact reported quarters unchanged. New top-down annual371.4301 implies FYQ4 126.5847 at revised Q3 102; own127 yields monthly bridge371.707. Fixed monthly weights cannot fully measure January redistribution; saved formulas/application recalculation, not pre-decision snapshot diagnostics, govern.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>